<commit_message>
paper run 2026-09-03 11:56
</commit_message>
<xml_diff>
--- a/reports/2026-09-03.xlsx
+++ b/reports/2026-09-03.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>-67.68000000000001</v>
+        <v>-44.16</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -647,43 +647,43 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-33.84</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>-33.84</v>
+        <v>8.1</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -692,33 +692,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-33.84</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>-33.84</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -737,163 +737,182 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>NO_LIQUIDITY</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n">
         <v>2</v>
       </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="n">
-        <v>-67.68000000000001</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="D24" t="n">
+        <v>-25.74</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>По окнам</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>По цене входа</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-09-03 17:56
</commit_message>
<xml_diff>
--- a/reports/2026-09-03.xlsx
+++ b/reports/2026-09-03.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,264 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-03T14:11:35.194269+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.00118</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-03T14:42:03.384540+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.0019</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-03T15:11:59.419834+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F4" t="n">
+        <v>32.79</v>
+      </c>
+      <c r="G4" t="n">
+        <v>61.87</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.0012</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>29.08</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-03T16:41:19.326369+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00168</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-03T17:11:46.269119+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F6" t="n">
+        <v>28.57</v>
+      </c>
+      <c r="G6" t="n">
+        <v>46.08</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00121</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>17.51</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-03T17:24:03.614984+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F7" t="n">
+        <v>35.36</v>
+      </c>
+      <c r="G7" t="n">
+        <v>69.34</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00107</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>33.98</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -527,7 +785,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -536,6 +794,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>0.8333333333333334</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>64.47</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>95.47</v>
       </c>
     </row>
     <row r="8">
@@ -564,7 +825,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-31</v>
       </c>
     </row>
     <row r="9">
@@ -573,6 +834,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>3.08</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>676.79</v>
+        <v>741.26</v>
       </c>
     </row>
     <row r="12">
@@ -632,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D15" t="n">
-        <v>-44.16</v>
+        <v>252.47</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>30.49</v>
       </c>
     </row>
     <row r="16">
@@ -651,16 +915,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" t="n">
-        <v>18.42</v>
+        <v>125.77</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>33.98</v>
       </c>
     </row>
     <row r="17">
@@ -673,180 +937,231 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>8.1</v>
+        <v>110.34</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>63.06</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>-33.84</v>
+        <v>65.06</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>17.51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>8</v>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-21</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D21" t="n">
-        <v>-33.84</v>
+        <v>122.04</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>9</v>
+      </c>
+      <c r="D23" t="n">
+        <v>254.16</v>
+      </c>
+      <c r="E23" t="n">
+        <v>77.95999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" t="n">
-        <v>2</v>
-      </c>
       <c r="D24" t="n">
-        <v>-25.74</v>
+        <v>55.31</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>68.77</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-13.49</v>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>83.17</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>13</v>
+      </c>
+      <c r="C28" t="n">
+        <v>11</v>
+      </c>
+      <c r="D28" t="n">
+        <v>180.85</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>114.22</v>
+      </c>
+      <c r="E29" t="n">
+        <v>64.47</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -855,67 +1170,383 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>63.06</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>17.51</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="n">
+        <v>30.49</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>33.98</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-21</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>29.08</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>51.49</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>77.95999999999999</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-13.49</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>73.06</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>17.51</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-26.1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>36.96</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" t="n">
+        <v>27.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-09-03 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-03.xlsx
+++ b/reports/2026-09-03.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -730,6 +730,92 @@
       </c>
       <c r="K7" t="n">
         <v>33.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-03T18:53:46.261997+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F8" t="n">
+        <v>37.06</v>
+      </c>
+      <c r="G8" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00147</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>35.61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-03T20:03:46.714140+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-0.00168</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>4.7</v>
       </c>
     </row>
   </sheetData>
@@ -743,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -765,7 +851,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -775,7 +861,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -795,7 +881,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="6">
@@ -805,7 +891,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64.47</v>
+        <v>104.78</v>
       </c>
     </row>
     <row r="7">
@@ -815,7 +901,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>95.47</v>
+        <v>135.78</v>
       </c>
     </row>
     <row r="8">
@@ -835,7 +921,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.08</v>
+        <v>4.38</v>
       </c>
     </row>
     <row r="10">
@@ -845,7 +931,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>741.26</v>
+        <v>781.5700000000001</v>
       </c>
     </row>
     <row r="12">
@@ -896,13 +982,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D15" t="n">
-        <v>252.47</v>
+        <v>419.42</v>
       </c>
       <c r="E15" t="n">
         <v>30.49</v>
@@ -915,16 +1001,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
-        <v>125.77</v>
+        <v>229.73</v>
       </c>
       <c r="E16" t="n">
-        <v>33.98</v>
+        <v>74.29000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -941,16 +1027,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>110.34</v>
+        <v>213.13</v>
       </c>
       <c r="E18" t="n">
-        <v>63.06</v>
+        <v>103.37</v>
       </c>
     </row>
     <row r="19">
@@ -960,13 +1046,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D19" t="n">
-        <v>65.06</v>
+        <v>169.8</v>
       </c>
       <c r="E19" t="n">
         <v>17.51</v>
@@ -979,13 +1065,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>80.8</v>
+        <v>114.7</v>
       </c>
       <c r="E20" t="n">
         <v>-21</v>
@@ -998,13 +1084,13 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
         <v>7</v>
       </c>
-      <c r="C21" t="n">
-        <v>6</v>
-      </c>
       <c r="D21" t="n">
-        <v>122.04</v>
+        <v>151.52</v>
       </c>
       <c r="E21" t="n">
         <v>4.9</v>
@@ -1024,16 +1110,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D23" t="n">
-        <v>254.16</v>
+        <v>495.59</v>
       </c>
       <c r="E23" t="n">
-        <v>77.95999999999999</v>
+        <v>118.27</v>
       </c>
     </row>
     <row r="24">
@@ -1043,13 +1129,13 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="n">
         <v>5</v>
       </c>
-      <c r="C24" t="n">
-        <v>4</v>
-      </c>
       <c r="D24" t="n">
-        <v>55.31</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1107,13 +1193,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C28" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D28" t="n">
-        <v>180.85</v>
+        <v>381.7</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -1126,16 +1212,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D29" t="n">
-        <v>114.22</v>
+        <v>184.28</v>
       </c>
       <c r="E29" t="n">
-        <v>64.47</v>
+        <v>104.78</v>
       </c>
     </row>
     <row r="31">
@@ -1174,13 +1260,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>63.06</v>
+        <v>103.37</v>
       </c>
     </row>
     <row r="35">
@@ -1276,13 +1362,13 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>33.98</v>
+        <v>74.29000000000001</v>
       </c>
     </row>
     <row r="43">
@@ -1371,182 +1457,214 @@
         <v>51.49</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>35.61</v>
+      </c>
+    </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>4</v>
-      </c>
-      <c r="C50" t="n">
-        <v>4</v>
-      </c>
-      <c r="D50" t="n">
-        <v>77.95999999999999</v>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>4.7</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" t="n">
-        <v>-13.49</v>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+      <c r="D52" t="n">
+        <v>118.27</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>3</v>
-      </c>
-      <c r="C54" t="n">
-        <v>3</v>
-      </c>
-      <c r="D54" t="n">
-        <v>73.06</v>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-13.49</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
-        <v>17.51</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>73.06</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
         <v>2</v>
       </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="n">
-        <v>-26.1</v>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>53.12</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" t="n">
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
         <v>3</v>
       </c>
-      <c r="D59" t="n">
-        <v>36.96</v>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-21.4</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" t="n">
+        <v>4</v>
+      </c>
+      <c r="D61" t="n">
+        <v>41.66</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B60" t="n">
-        <v>2</v>
-      </c>
-      <c r="C60" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" t="n">
-        <v>27.51</v>
+      <c r="B62" t="n">
+        <v>3</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>63.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>